<commit_message>
Update 001/SV-P Pikachu watchlist row with overseas price and downtrend
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFJb2XBSW3qiXZccuwfJhv
</commit_message>
<xml_diff>
--- a/import_calculator.xlsx
+++ b/import_calculator.xlsx
@@ -2245,11 +2245,142 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2026/8/12</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">低単価で練習向き。取引数が多く売りやすい</t>
+      <t xml:space="preserve">2026/9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ヶ月前</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16,500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PSA10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">が約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万枚と多く下落中。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">eBay</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">出品は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">57</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">107</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ドルで上限超え</t>
+    </r>
   </si>
   <si>
     <r>
@@ -5427,7 +5558,7 @@
         <v>110</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>20</v>
@@ -5436,12 +5567,14 @@
         <f aca="false">IF(D21="","",MAX(0,ROUNDDOWN(((D21*(1-設定!$B$11)-設定!$B$12-設定!$B$10-MAX(D21*設定!$B$14,設定!$B$13))/(1+設定!$B$6+設定!$B$7+設定!$B$8*(1+設定!$B$7)))/設定!$B$5-G21,0)))</f>
         <v>35</v>
       </c>
-      <c r="I21" s="13"/>
+      <c r="I21" s="13" t="n">
+        <v>57</v>
+      </c>
       <c r="J21" s="5" t="str">
         <f aca="false">IF(I21="","要調査（eBayで確認）",IF(I21&lt;=H21,"平均でも利益あり","割安出品を待つ"))</f>
-        <v>要調査（eBayで確認）</v>
-      </c>
-      <c r="K21" s="5" t="s">
+        <v>割安出品を待つ</v>
+      </c>
+      <c r="K21" s="9" t="s">
         <v>111</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add English-version card research and Iono promo to watchlist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFJb2XBSW3qiXZccuwfJhv
</commit_message>
<xml_diff>
--- a/import_calculator.xlsx
+++ b/import_calculator.xlsx
@@ -372,7 +372,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="186">
   <si>
     <t xml:space="preserve">輸入型 仕入れ判定ツール — 設定</t>
   </si>
@@ -2196,6 +2196,165 @@
   </si>
   <si>
     <t xml:space="preserve">海外相場の方が高い。日本限定でも逆転している例</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ナンジャモ 英語版プロモ（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Iono</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SVP EN 124</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ポケカチ相場</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">26,200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円・店頭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">23,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">27,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円（出品価格。低めに採用）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">英語版のみ。キャラ人気で日本に</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PSA10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の上乗せあり。資金</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円台では</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">45</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ドル以下の出品待ち</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4881,7 +5040,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -5552,49 +5711,71 @@
         <v>43</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>14300</v>
+        <v>22000</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>110</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H21" s="14" t="n">
         <f aca="false">IF(D21="","",MAX(0,ROUNDDOWN(((D21*(1-設定!$B$11)-設定!$B$12-設定!$B$10-MAX(D21*設定!$B$14,設定!$B$13))/(1+設定!$B$6+設定!$B$7+設定!$B$8*(1+設定!$B$7)))/設定!$B$5-G21,0)))</f>
-        <v>35</v>
+        <v>77</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="J21" s="5" t="str">
         <f aca="false">IF(I21="","要調査（eBayで確認）",IF(I21&lt;=H21,"平均でも利益あり","割安出品を待つ"))</f>
         <v>割安出品を待つ</v>
       </c>
-      <c r="K21" s="9" t="s">
+      <c r="K21" s="5" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
+      <c r="A22" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>14300</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <f aca="false">IF(D22="","",MAX(0,ROUNDDOWN(((D22*(1-設定!$B$11)-設定!$B$12-設定!$B$10-MAX(D22*設定!$B$14,設定!$B$13))/(1+設定!$B$6+設定!$B$7+設定!$B$8*(1+設定!$B$7)))/設定!$B$5-G22,0)))</f>
+        <v>35</v>
+      </c>
+      <c r="I22" s="13" t="n">
+        <v>57</v>
+      </c>
+      <c r="J22" s="5" t="str">
+        <f aca="false">IF(I22="","要調査（eBayで確認）",IF(I22&lt;=H22,"平均でも利益あり","割安出品を待つ"))</f>
+        <v>割安出品を待つ</v>
+      </c>
+      <c r="K22" s="9" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>112</v>
-      </c>
+      <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -5608,7 +5789,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -5621,8 +5802,23 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J5:J21">
+  <conditionalFormatting sqref="J5:J22">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>J5="平均でも利益あり"</formula>
     </cfRule>
@@ -5672,69 +5868,69 @@
         <v>30</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N1" s="11" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="O1" s="11" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P1" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="R1" s="11" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="S1" s="11" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D2" s="13" t="n">
         <v>180</v>
@@ -5749,7 +5945,7 @@
         <v>45000</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="I2" s="17" t="n">
         <f aca="false">IF(D2="","",(D2+E2)*設定!$B$5*(1+設定!$B$6)+F2)</f>
@@ -7385,7 +7581,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -7448,7 +7644,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7456,7 +7652,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7470,7 +7666,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D3" s="2"/>
     </row>
@@ -7483,74 +7679,74 @@
         <v>100000</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>6000</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>30000</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>30</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">ROUNDUP(B4/B5,0)</f>
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B10" s="23" t="n">
         <f aca="false">B9/30</f>
@@ -7561,40 +7757,40 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B11" s="17" t="n">
         <f aca="false">B9*B6</f>
         <v>510000</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B12" s="24" t="n">
         <f aca="false">ROUNDUP(B11*MAX(B7,1)/30*(1+B8),-4)</f>
         <v>620000</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">B9*(B6+B5)</f>
         <v>612000</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D13" s="2"/>
     </row>
@@ -7612,7 +7808,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -7620,21 +7816,21 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>10000</v>
@@ -7644,12 +7840,12 @@
         <v>2</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>30000</v>
@@ -7659,12 +7855,12 @@
         <v>5</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>60000</v>
@@ -7674,12 +7870,12 @@
         <v>10</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B21" s="8" t="n">
         <v>100000</v>
@@ -7689,7 +7885,7 @@
         <v>17</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -7726,10 +7922,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C1" s="27" t="s">
         <v>30</v>
@@ -7741,38 +7937,38 @@
         <v>32</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="I1" s="27" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="J1" s="27" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="K1" s="27" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="L1" s="27" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="M1" s="27" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="N1" s="27" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="O1" s="27" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="P1" s="2"/>
       <c r="Q1" s="25" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="R1" s="28" t="n">
         <f aca="false">SUM(L2:L101)</f>
@@ -7787,19 +7983,19 @@
         <v>46285</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D2" s="30" t="s">
         <v>43</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H2" s="31" t="n">
         <v>36294</v>
@@ -7828,11 +8024,11 @@
         <v>19</v>
       </c>
       <c r="O2" s="12" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="25" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="R2" s="32" t="n">
         <f aca="false">COUNT(L2:L101)</f>
@@ -7872,7 +8068,7 @@
       <c r="O3" s="30"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="25" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="R3" s="28" t="n">
         <f aca="false">IFERROR(AVERAGE(L2:L101),0)</f>
@@ -7912,7 +8108,7 @@
       <c r="O4" s="30"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="25" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="R4" s="32" t="n">
         <f aca="false">IFERROR(AVERAGE(N2:N101),0)</f>

</xml_diff>

<commit_message>
Record opened pack cost in trade log and add unrecovered-cost summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFJb2XBSW3qiXZccuwfJhv
</commit_message>
<xml_diff>
--- a/import_calculator.xlsx
+++ b/import_calculator.xlsx
@@ -371,8 +371,42 @@
 </comments>
 </file>
 
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="Q5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">販売価格が空欄の行（パック代など、まだ売れていない仕入れ）の原価合計</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">合計利益から未販売の原価を引いた、今の手取りベースの利益</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="190">
   <si>
     <t xml:space="preserve">輸入型 仕入れ判定ツール — 設定</t>
   </si>
@@ -4108,50 +4142,55 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">鑑定品</t>
-  </si>
-  <si>
-    <t xml:space="preserve">メルカリ</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">海外</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30th CELEBRATION 15</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Sold</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パック＋ストームエメラルダ </t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">より国内相場が高く、</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">PSA</t>
-    </r>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パック（開封）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">パック</t>
+  </si>
+  <si>
+    <t xml:space="preserve">店頭（定価）</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -4159,7 +4198,178 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">証明番号で真贋確認済み</t>
+      <t xml:space="preserve">原価</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 30th 360</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×15=5,400</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円＋ストームエメラルダ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">180</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×6=1,080</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パック</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">180</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円は仮。要確認）。仕入日は仮。開封分</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">39</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">枚は売れたら下の行に原価</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円で記録し、合計からこの</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6,480</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円を引く</t>
     </r>
   </si>
   <si>
@@ -4207,6 +4417,86 @@
   </si>
   <si>
     <t xml:space="preserve">平均在庫日数</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">未販売の原価</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">実質利益</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -7972,67 +8262,61 @@
       </c>
       <c r="R1" s="28" t="n">
         <f aca="false">SUM(L2:L101)</f>
-        <v>6676</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="n">
-        <v>46266</v>
-      </c>
-      <c r="B2" s="29" t="n">
-        <v>46285</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>135</v>
+        <v>46290</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="30" t="s">
+        <v>180</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>43</v>
+        <v>181</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>181</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="G2" s="30"/>
       <c r="H2" s="31" t="n">
-        <v>36294</v>
-      </c>
-      <c r="I2" s="31" t="n">
-        <v>48000</v>
-      </c>
-      <c r="J2" s="17" t="n">
+        <v>6480</v>
+      </c>
+      <c r="I2" s="31"/>
+      <c r="J2" s="17" t="str">
         <f aca="false">IF(I2="","",ROUNDDOWN(I2*設定!$B$11,0))</f>
-        <v>4800</v>
-      </c>
-      <c r="K2" s="17" t="n">
+        <v/>
+      </c>
+      <c r="K2" s="17" t="str">
         <f aca="false">IF(I2="","",設定!$B$12)</f>
-        <v>230</v>
-      </c>
-      <c r="L2" s="17" t="n">
+        <v/>
+      </c>
+      <c r="L2" s="17" t="str">
         <f aca="false">IF(OR(H2="",I2=""),"",I2-H2-J2-K2)</f>
-        <v>6676</v>
-      </c>
-      <c r="M2" s="18" t="n">
+        <v/>
+      </c>
+      <c r="M2" s="18" t="str">
         <f aca="false">IF(OR(L2="",I2=0),"",L2/I2)</f>
-        <v>0.139083333333333</v>
-      </c>
-      <c r="N2" s="5" t="n">
+        <v/>
+      </c>
+      <c r="N2" s="5" t="str">
         <f aca="false">IF(OR(A2="",B2=""),"",B2-A2)</f>
-        <v>19</v>
+        <v/>
       </c>
       <c r="O2" s="12" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="25" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="R2" s="32" t="n">
         <f aca="false">COUNT(L2:L101)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8068,11 +8352,11 @@
       <c r="O3" s="30"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="25" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="R3" s="28" t="n">
         <f aca="false">IFERROR(AVERAGE(L2:L101),0)</f>
-        <v>6676</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8108,11 +8392,11 @@
       <c r="O4" s="30"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="25" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="R4" s="32" t="n">
         <f aca="false">IFERROR(AVERAGE(N2:N101),0)</f>
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8147,8 +8431,13 @@
       </c>
       <c r="O5" s="30"/>
       <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
+      <c r="Q5" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="R5" s="28" t="n">
+        <f aca="false">SUMIFS(H2:H101,I2:I101,"")</f>
+        <v>6480</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29"/>
@@ -8182,8 +8471,13 @@
       </c>
       <c r="O6" s="30"/>
       <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
+      <c r="Q6" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="R6" s="28" t="n">
+        <f aca="false">R1-R5</f>
+        <v>-6480</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29"/>
@@ -11518,5 +11812,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>